<commit_message>
Updated the Single Ton class pattern's need to implement them
</commit_message>
<xml_diff>
--- a/src/test/resources/Data.xlsx
+++ b/src/test/resources/Data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kspraneeth\Desktop\Important\main code\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44986368-213F-4E91-AE51-0F1D6AE453CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DD7E031-AB8D-44BF-8E88-43B1CEBEC2ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="39">
   <si>
     <t>TestCaseNo</t>
   </si>
@@ -133,6 +133,15 @@
   </si>
   <si>
     <t>adg</t>
+  </si>
+  <si>
+    <t>execution flag</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>N</t>
   </si>
 </sst>
 </file>
@@ -498,15 +507,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.77734375" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="16384" width="8.88671875" style="2"/>
+    <col min="3" max="3" width="13.33203125" style="2" customWidth="1"/>
+    <col min="4" max="16384" width="8.88671875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -514,19 +524,22 @@
         <v>1</v>
       </c>
       <c r="C1" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="F1" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="G1" s="6" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>19</v>
       </c>
@@ -534,19 +547,22 @@
         <v>4</v>
       </c>
       <c r="C2" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="F2" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="G2" s="4" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>20</v>
       </c>
@@ -554,19 +570,22 @@
         <v>5</v>
       </c>
       <c r="C3" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="F3" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="G3" s="4" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>21</v>
       </c>
@@ -574,19 +593,22 @@
         <v>6</v>
       </c>
       <c r="C4" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="F4" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="G4" s="4" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>22</v>
       </c>
@@ -594,19 +616,22 @@
         <v>7</v>
       </c>
       <c r="C5" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="F5" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="G5" s="4" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>23</v>
       </c>
@@ -614,15 +639,18 @@
         <v>8</v>
       </c>
       <c r="C6" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="E6" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="F6" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="G6" s="4" t="s">
         <v>35</v>
       </c>
     </row>

</xml_diff>